<commit_message>
Add GHRU-backed QC and manuscript reporting
</commit_message>
<xml_diff>
--- a/examples/qualibact_ecoli/fail_only/report/report.xlsx
+++ b/examples/qualibact_ecoli/fail_only/report/report.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC3"/>
+  <dimension ref="A1:AI3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -489,82 +489,112 @@
       </c>
       <c r="N1" t="inlineStr">
         <is>
+          <t>Checkm.Total_Coding_Sequences</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
           <t>Checkm.all_checks_passed</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Quast.# contigs (&gt;= 0 bp)</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Quast.GC (%)</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>Quast.Largest contig</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Quast.N50</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>Quast.Total length</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Quast.Total length (&gt;= 0 bp)</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>Quast.all_checks_passed</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>Speciator.all_checks_passed</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>Speciator.confidence</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>Speciator.speciesName</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>Sylph.all_checks_passed</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>Sylph.number_of_genomes</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>Sylph.top_species</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>Sylph.top_taxonomic_abundance</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>all_checks_passed</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
+          <t>qualibact_compat_tier</t>
+        </is>
+      </c>
+      <c r="AF1" t="inlineStr">
+        <is>
+          <t>qualibact_compat_passed</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>qualibact_compat_reasons</t>
+        </is>
+      </c>
+      <c r="AH1" t="inlineStr">
+        <is>
+          <t>qualibact_compat_warn_policy</t>
+        </is>
+      </c>
+      <c r="AI1" t="inlineStr">
+        <is>
+          <t>qualibact_compat_source</t>
         </is>
       </c>
     </row>
@@ -574,23 +604,35 @@
           <t>SAMD00006077</t>
         </is>
       </c>
-      <c r="B2" t="b">
-        <v>1</v>
-      </c>
-      <c r="C2" t="b">
-        <v>1</v>
-      </c>
-      <c r="D2" t="b">
-        <v>1</v>
-      </c>
-      <c r="E2" t="b">
-        <v>0</v>
-      </c>
-      <c r="F2" t="b">
-        <v>0</v>
-      </c>
-      <c r="G2" t="b">
-        <v>0</v>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
       </c>
       <c r="H2" t="n">
         <v>522</v>
@@ -610,59 +652,97 @@
       <c r="M2" t="n">
         <v>19474</v>
       </c>
-      <c r="N2" t="b">
-        <v>0</v>
-      </c>
-      <c r="O2" t="n">
+      <c r="N2" t="n">
+        <v>4264</v>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="P2" t="n">
         <v>522</v>
       </c>
-      <c r="P2" t="n">
+      <c r="Q2" t="n">
         <v>50.8872</v>
       </c>
-      <c r="Q2" t="n">
+      <c r="R2" t="n">
         <v>69909</v>
       </c>
-      <c r="R2" t="n">
+      <c r="S2" t="n">
         <v>19474</v>
-      </c>
-      <c r="S2" t="n">
-        <v>4153626</v>
       </c>
       <c r="T2" t="n">
         <v>4153626</v>
       </c>
-      <c r="U2" t="b">
-        <v>0</v>
-      </c>
-      <c r="V2" t="b">
+      <c r="U2" t="n">
+        <v>4153626</v>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>Escherichia coli</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="AA2" t="n">
         <v>1</v>
       </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
-      <c r="X2" t="inlineStr">
+      <c r="AB2" t="inlineStr">
         <is>
           <t>Escherichia coli</t>
         </is>
       </c>
-      <c r="Y2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Z2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA2" t="inlineStr">
-        <is>
-          <t>Escherichia coli</t>
-        </is>
-      </c>
-      <c r="AB2" t="n">
+      <c r="AC2" t="n">
         <v>0.75</v>
       </c>
-      <c r="AC2" t="b">
-        <v>0</v>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="AG2" t="inlineStr">
+        <is>
+          <t>N50 &lt;20000.0; GC_Content &gt;50.88; Genome_Size &lt;4400000.0</t>
+        </is>
+      </c>
+      <c r="AH2" t="inlineStr">
+        <is>
+          <t>warn-as-warn</t>
+        </is>
+      </c>
+      <c r="AI2" t="inlineStr">
+        <is>
+          <t>QualiBact Escherichia_coli qualibact-v1.0 ATB tier logic</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -671,23 +751,35 @@
           <t>SAMN42765982</t>
         </is>
       </c>
-      <c r="B3" t="b">
-        <v>1</v>
-      </c>
-      <c r="C3" t="b">
-        <v>1</v>
-      </c>
-      <c r="D3" t="b">
-        <v>0</v>
-      </c>
-      <c r="E3" t="b">
-        <v>1</v>
-      </c>
-      <c r="F3" t="b">
-        <v>1</v>
-      </c>
-      <c r="G3" t="b">
-        <v>0</v>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
       </c>
       <c r="H3" t="n">
         <v>679</v>
@@ -707,59 +799,97 @@
       <c r="M3" t="n">
         <v>126621</v>
       </c>
-      <c r="N3" t="b">
-        <v>0</v>
-      </c>
-      <c r="O3" t="n">
+      <c r="N3" t="n">
+        <v>6105</v>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="P3" t="n">
         <v>679</v>
       </c>
-      <c r="P3" t="n">
+      <c r="Q3" t="n">
         <v>50.5585</v>
       </c>
-      <c r="Q3" t="n">
+      <c r="R3" t="n">
         <v>312707</v>
       </c>
-      <c r="R3" t="n">
+      <c r="S3" t="n">
         <v>126621</v>
-      </c>
-      <c r="S3" t="n">
-        <v>5738641</v>
       </c>
       <c r="T3" t="n">
         <v>5738641</v>
       </c>
-      <c r="U3" t="b">
-        <v>0</v>
-      </c>
-      <c r="V3" t="b">
+      <c r="U3" t="n">
+        <v>5738641</v>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>Escherichia coli</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="AA3" t="n">
         <v>1</v>
       </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
-      <c r="X3" t="inlineStr">
+      <c r="AB3" t="inlineStr">
         <is>
           <t>Escherichia coli</t>
         </is>
       </c>
-      <c r="Y3" t="b">
-        <v>1</v>
-      </c>
-      <c r="Z3" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA3" t="inlineStr">
-        <is>
-          <t>Escherichia coli</t>
-        </is>
-      </c>
-      <c r="AB3" t="n">
+      <c r="AC3" t="n">
         <v>0.75</v>
       </c>
-      <c r="AC3" t="b">
-        <v>0</v>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="AF3" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="AG3" t="inlineStr">
+        <is>
+          <t>no_of_contigs &gt;670.0; Genome_Size &gt;5700000.0; Total_Coding_Sequences &gt;5800.0</t>
+        </is>
+      </c>
+      <c r="AH3" t="inlineStr">
+        <is>
+          <t>warn-as-warn</t>
+        </is>
+      </c>
+      <c r="AI3" t="inlineStr">
+        <is>
+          <t>QualiBact Escherichia_coli qualibact-v1.0 ATB tier logic</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -898,7 +1028,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -983,12 +1113,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Sylph.top_species</t>
+          <t>qualibact_compat_tier</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Escherichia coli</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -1004,25 +1134,46 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Sylph.top_taxonomic_abundance</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
+          <t>Sylph.top_species</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Escherichia coli</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
       <c r="D5" t="n">
         <v>0</v>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Sylph.top_taxonomic_abundance</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="inlineStr">
         <is>
           <t>0.75</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>0.75</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>0.75</t>
         </is>

</xml_diff>